<commit_message>
Hydro-AF-NAVY-Converter - Cutler Conversion - updating hydro script to newest changes, adding InstallationIDs to Installation_IDs excel file
</commit_message>
<xml_diff>
--- a/Installation_IDs.xlsx
+++ b/Installation_IDs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\RStor\CEMML\ClimateChange\Document Standards\Templates\TEMPLATES_SME_Word_Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\C838011553\Documents\Converter Code\GIT\HTML-Converter-RScripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3900F204-82F0-4007-B7F0-AB0ACFBA2B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45148317-81BB-4636-AEEF-36A30154ACDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AIR FORCE" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="111">
   <si>
     <t>SITEID</t>
   </si>
@@ -335,13 +335,37 @@
   </si>
   <si>
     <t>Naval Submarine Base Kings Bay</t>
+  </si>
+  <si>
+    <t>InstallationID</t>
+  </si>
+  <si>
+    <t>N62688</t>
+  </si>
+  <si>
+    <t>N42237</t>
+  </si>
+  <si>
+    <t>N69212</t>
+  </si>
+  <si>
+    <t>N61008</t>
+  </si>
+  <si>
+    <t>N00207</t>
+  </si>
+  <si>
+    <t>N60201</t>
+  </si>
+  <si>
+    <t>N32446-LF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -374,6 +398,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -392,9 +421,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -404,9 +434,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{0CA8EF0B-0BDB-4DAF-B59A-3C1C782D2818}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{7F1440B0-8B00-42F4-9304-B99C2DA4E6E1}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1455,80 +1486,106 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A06A16C-6F98-439D-96DD-17D8D49F3FE1}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="41.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>